<commit_message>
docs(visio): detalhar fluxograma real do painel do vendedor
Adiciona o ciclo E2E sequencial (auth, KYC, loja, overview, listing,
estoque, pedidos, fulfillment, $) e abas por módulo com APIs e gates.

Co-authored-by: Guilherme Cardoso <guibruno93@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/architecture/visio/JudgeTCG_Painel_Vendedor_Investidor.xlsx
+++ b/docs/architecture/visio/JudgeTCG_Painel_Vendedor_Investidor.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Modulos_Investidor" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Como_importar_Visio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="F01_Ciclo_E2E" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -149,6 +150,21 @@
     <tableColumn id="5" name="Sem FastAPI/Render"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="F01CicloE2E" displayName="F01CicloE2E" ref="A1:F30" headerRowCount="1">
+  <autoFilter ref="A1:F30"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Process Step ID"/>
+    <tableColumn id="2" name="Process Step Description"/>
+    <tableColumn id="3" name="Next Step ID"/>
+    <tableColumn id="4" name="Connector Label"/>
+    <tableColumn id="5" name="Shape Type"/>
+    <tableColumn id="6" name="Function / Area"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
 </table>
 </file>
 
@@ -1113,7 +1129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1183,16 +1199,933 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fonte de UI: frontend/runtime_console_v3/src/lib/seller-sidebar-nav.ts</t>
+          <t>Abas novas do .vsdx: Ciclo E2E (fluxograma mestre), Dashboard, Operação Inbox, Catálogo, Estoque, Pedidos, Financeiro, Marketing CRM, Equipe PDV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Abas F01_Ciclo_E2E neste Excel: Visualizador de Dados (Passo ID → próximo).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Process Step ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Process Step Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Next Step ID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Connector Label</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Shape Type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Function / Area</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Lojista quer vender no JudgeTCG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GET /entrar · Supabase Auth</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HTTPS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>External Data</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sessão JWT?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>E03;E04</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Não;Sim</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Redirect /entrar?next=painel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GET /api/account/status KYC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HTTP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>External Data</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FastAPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Status leu?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>E06;E07</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>503;Sim</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Banner status indisponível (fail-open)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>can_publish / KYC ok?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>E08;E09</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Não;Sim</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>KYC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GET /loja/suspensa</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>KYC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GET /api/stores/mine</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>HTTP</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Há loja?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>E11;E13</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Não;Sim</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>POST /api/stores /stores/create + CNPJ</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>E12;E13</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>POST Stripe Connect onboard</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HTTPS</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>External Data</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>GET /api/seller/dashboard/overview</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HTTP</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Overview 200?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>E15;E16</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Não;Sim</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mock KPIs pending_payment=12 tickets=3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Catálogo GET cartas/produtos/jogos</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>POST /api/seller/listings wizard</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>E18;E19</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Listagens</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>POST /api/seller/inventory/*</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Estoque</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Buyer vê PDP / listing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Checkout Stripe ou PIX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HTTPS</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>External Data</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pedido SQL marketplace</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GET /api/seller/orders + tabs</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>E23;E24</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>POST bulk/fulfillment/commands</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Fulfillment</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GET /api/seller/tickets</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Atendimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Repasse Stripe Connect / PIX</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Subprocess</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Financeiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LPC sem equipe JudgeTCG?</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>E27;E28</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ainda não;quando houver evidência</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>North Star</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LPC = 0 Beta not started</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Ciclo de produto desenhado</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>